<commit_message>
Homework: add ROC step with live chart (week2) and scree plot chart (week6)
- week2 Step5_ROC: TPR/FPR at three thresholds, trapezoid AUC (=0.74), and
  a scatter chart wired to the student's answer cells so the ROC curve
  draws itself as the yellow cells are filled
- week6 Step3: line chart of PVE and cumulative PVE (scree plot), also fed
  by the student's own answers
- verified: recalc zero errors; fill-answers self-test passes (now 212
  checks); charts confirmed rendering with filled answers
</commit_message>
<xml_diff>
--- a/week2/homework-regression-classification.xlsx
+++ b/week2/homework-regression-classification.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Step2_Inference" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Step3_Logistic" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Step4_Confusion" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Answer_Key" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Step5_ROC" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Answer_Key" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="173">
   <si>
     <t xml:space="preserve">[Description] Regression &amp; Classification</t>
   </si>
@@ -363,6 +364,75 @@
     <t xml:space="preserve">think about which error you trade away</t>
   </si>
   <si>
+    <t xml:space="preserve">[Description] STEP 5: trace the ROC curve from three thresholds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One curve, every threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISLP §4.4.2 · Week 2 slide "The ROC curve: all thresholds at once"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same 10 cases as Step 4 (5 true positives, 5 true negatives). Predict ŷ=1 when p̂ ≥ t.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIVEN: the ten cases again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill TP, FP, then TPR = TP/5 and FPR = FP/5 at each threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">threshold t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plot data (auto-fills from your answers above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FPR (x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPR (y)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t=1 (reject all)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t=0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t=0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t=0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t=0 (accept all)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area under your 5-point curve (trapezoids) =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Σ (x₂-x₁)·(y₁+y₂)/2 over the 4 segments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A useless classifier has AUC =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the diagonal</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Description] ANSWER KEY - all solutions. No peeking until you have tried!</t>
   </si>
   <si>
@@ -460,6 +530,21 @@
   </si>
   <si>
     <t xml:space="preserve">Lower threshold raises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STEP 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(FPR, TPR) at t=0.75 / 0.5 / 0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0, 0.4), (0.2, 0.6), (0.6, 0.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUC (trapezoid, 5 points)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Useless classifier AUC</t>
   </si>
 </sst>
 </file>
@@ -469,7 +554,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,6 +627,26 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -565,7 +670,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD8E4BC"/>
-        <bgColor rgb="FFDAEEF3"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -621,7 +726,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -674,6 +779,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -714,7 +823,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF2F2F2"/>
@@ -722,7 +831,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF1E64C8"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -741,7 +850,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF4472C4"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF98B855"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -758,6 +867,640 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:style val="13"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1800" b="1" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Your ROC curve</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"ROC"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ROC</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="98B855"/>
+            </a:solidFill>
+            <a:ln w="12600">
+              <a:solidFill>
+                <a:srgbClr val="98B855"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98B855"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="12600">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                </a:ln>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Step5_ROC!$B$32:$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Step5_ROC!$C$32:$C$36</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:axId val="74388445"/>
+        <c:axId val="52950048"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="74388445"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr sz="1000" b="1" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>False positive rate</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="52950048"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="52950048"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr sz="1000" b="1" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:uFillTx/>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>True positive rate</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:uFillTx/>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="74388445"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:uFillTx/>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>398880</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>170640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5356800" y="4572000"/>
+        <a:ext cx="4679640" cy="3599640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2195,7 +2938,363 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="5" t="str">
+        <f aca="false">IF(COUNT(B26:E26)=0,"",IF(AND(ROUND(B26,3)=ROUND(2,3),ROUND(C26,3)=ROUND(0,3),ROUND(D26,3)=ROUND(0.4,3),ROUND(E26,3)=ROUND(0,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="5" t="str">
+        <f aca="false">IF(COUNT(B27:E27)=0,"",IF(AND(ROUND(B27,3)=ROUND(3,3),ROUND(C27,3)=ROUND(1,3),ROUND(D27,3)=ROUND(0.6,3),ROUND(E27,3)=ROUND(0.2,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="5" t="str">
+        <f aca="false">IF(COUNT(B28:E28)=0,"",IF(AND(ROUND(B28,3)=ROUND(4,3),ROUND(C28,3)=ROUND(3,3),ROUND(D28,3)=ROUND(0.8,3),ROUND(E28,3)=ROUND(0.6,3)),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <f aca="false">E26</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <f aca="false">D26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B34" s="6" t="n">
+        <f aca="false">E27</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <f aca="false">D27</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B35" s="6" t="n">
+        <f aca="false">E28</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <f aca="false">D28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" s="11"/>
+      <c r="F38" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G38" s="12"/>
+      <c r="H38" s="5" t="str">
+        <f aca="false">IF(G38="","",IF(ROUND(G38,3)=ROUND(0.74,3),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E40" s="11"/>
+      <c r="F40" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G40" s="12"/>
+      <c r="H40" s="5" t="str">
+        <f aca="false">IF(G40="","",IF(ROUND(G40,3)=ROUND(0.5,3),"✓","✗"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D40:E40"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A1:J40">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"✓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"✗"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -2204,30 +3303,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>10</v>
@@ -2235,7 +3334,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>14</v>
@@ -2243,7 +3342,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>1.4</v>
@@ -2251,7 +3350,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>2.8</v>
@@ -2259,28 +3358,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B17" s="7" t="n">
         <v>0.4</v>
@@ -2296,7 +3395,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>0.1155</v>
@@ -2312,7 +3411,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>20</v>
@@ -2328,36 +3427,36 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B29" s="7" t="n">
         <v>7.389</v>
@@ -2365,7 +3464,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B30" s="7" t="n">
         <v>2</v>
@@ -2373,20 +3472,20 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B35" s="7" t="n">
         <v>0.7</v>
@@ -2394,7 +3493,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="B36" s="7" t="n">
         <v>0.6</v>
@@ -2402,7 +3501,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="B37" s="7" t="n">
         <v>0.8</v>
@@ -2410,10 +3509,39 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>142</v>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>